<commit_message>
Upload Week 4 & 5
</commit_message>
<xml_diff>
--- a/AI_Audit-Log_DE190359.xlsx
+++ b/AI_Audit-Log_DE190359.xlsx
@@ -1,28 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT\Sem 7\SWD392\AI Audit Log\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4EE26BC-1C63-45AA-B98C-7DF074FE5D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BAC22CD-B5F3-4475-AACE-B1C143295BCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 1 " sheetId="1" r:id="rId1"/>
     <sheet name="Week 2" sheetId="2" r:id="rId2"/>
     <sheet name="Week 3" sheetId="4" r:id="rId3"/>
+    <sheet name="Week 4 " sheetId="5" r:id="rId4"/>
+    <sheet name="Week 5" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="128">
   <si>
     <t>STT</t>
   </si>
@@ -333,6 +335,114 @@
   <si>
     <t>Phản hồi: AI đề xuất checklist 6 điểm: (1) Có đủ lifeline đại diện cho tất cả layer không; (2) Alt fragment có guard condition rõ ràng và lồng đúng logic không; (3) Mỗi synchronous call có return message tương ứng không; (4) Repository Pattern đúng – không có message nào đi thẳng đến Database; (5) Thứ tự lifeline từ trái sang phải theo luồng xử lý; (6) Tên method khớp với ngôn ngữ domain.
 Quyết định: Tôi bổ sung thêm 3 mục từ lỗi thực tế tôi vừa sửa: (7) Kiểm tra fragment thanh toán nằm bên trong nhánh [car available], không tách riêng; (8) PaymentService không gọi thẳng BookingRepository – vi phạm Single Responsibility; (9) Có đủ message updateStatus() sau các bước tạo booking và xử lý thanh toán. Ba điểm này tôi ghi nhớ rất rõ vì vừa mắc phải.</t>
+  </si>
+  <si>
+    <t>"Sequence diagram là gì, dùng để làm gì trong phân tích thiết kế hệ thống?"</t>
+  </si>
+  <si>
+    <t>"Một sequence diagram bao gồm những phần tử cơ bản nào? Giải thích ý nghĩa từng phần."</t>
+  </si>
+  <si>
+    <t>"Phân biệt alt, opt và loop trong sequence diagram, minh họa bằng hệ thống AutoGo."</t>
+  </si>
+  <si>
+    <t>"Vẽ sequence diagram cho use case 'Create Booking and Pay Deposit' của AutoGo theo kiến trúc phân lớp. Cần những lifeline nào?"</t>
+  </si>
+  <si>
+    <t>"Trong sequence diagram của AutoGo, hai khối alt cần có nằm ở đâu và điều kiện rẽ nhánh là gì?"</t>
+  </si>
+  <si>
+    <t>"Cách thể hiện Repository Pattern cho rõ trong sequence diagram? Quy ước đặt tên method ra sao?"</t>
+  </si>
+  <si>
+    <t>"Sequence diagram cho use case 'Return Car' cần thể hiện gì? Staff và hệ thống tương tác như thế nào?"</t>
+  </si>
+  <si>
+    <t>"Khi nào dùng &lt;&lt;boundary&gt;&gt;, &lt;&lt;control&gt;&gt;, &lt;&lt;entity&gt;&gt; trong sequence diagram theo mô hình MVC/Layered? Áp dụng vào AutoGo ra sao?"</t>
+  </si>
+  <si>
+    <t>"Trước khi nộp bài SWD392, cần checklist gì để tự kiểm tra sequence diagram của AutoGo?"</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Đây là một loại biểu đồ hành vi trong UML, dùng để minh họa các đối tượng trao đổi thông điệp với nhau theo dòng thời gian — cho biết đối tượng nào gọi đối tượng nào và theo thứ tự ra sao. Vai trò chính là mô tả luồng xử lý cho một use case nhất định. Đánh giá: Nội dung chính xác, đầy đủ. Em bổ sung thêm sự khác biệt với collaboration diagram: cả hai đều thể hiện tương tác nhưng sequence diagram tập trung vào yếu tố thời gian, còn collaboration diagram tập trung vào cấu trúc các quan hệ — điều này AI chưa nhắc tới.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Các thành phần gồm: lifeline (đại diện actor/object), activation bar, các loại message (đồng bộ, bất đồng bộ, message trả về), và combined fragment (alt, loop, opt, ref), cùng các stereotype boundary/control/entity. Đánh giá: Khớp với chuẩn UML 2.x. Tuy nhiên AI chưa làm rõ cách vẽ mũi tên phân biệt message đồng bộ (đầu mũi tên đặc) và bất đồng bộ (đầu mũi tên hở) — em tự ghi chú lại quy ước này để áp dụng đúng khi vẽ trên PlantUML.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: alt thể hiện rẽ nhánh có điều kiện (tương tự if-else), opt là khối chỉ thực thi khi thỏa điều kiện (giống if không có else), loop là khối lặp. Ví dụ trong AutoGo: dùng alt [xe còn trống]/[hết xe] ngay sau checkAvailability(); dùng opt [xe có hư hỏng] sau bước kiểm tra xe; dùng loop [mỗi lần thanh toán] khi khách trả góp nhiều lần. Đánh giá: Các ví dụ gắn sát với bài toán AutoGo, rất hữu ích. Em giữ nguyên 3 ví dụ này để làm mẫu tham khảo khi luyện vẽ diagram.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Đề xuất các lifeline: Customer, BookingUI, BookingController, CarRepository, BookingRepository, PaymentService, PaymentRepository. Luồng xử lý: khách hàng gửi yêu cầu → UI chuyển tới Controller → Controller gọi CarRepository.checkAvailability() → trong alt [còn xe] gọi BookingRepository.save() → tiếp tục PaymentService.processDeposit() → PaymentRepository.save() → phản hồi kết quả về UI. Đánh giá: Về cơ bản đủ các lớp, đúng hướng. Tuy nhiên em rà lại thấy Controller không nên gọi trực tiếp xuống Repository mà phải qua Service — em chỉnh lại thành BookingController → BookingService → BookingRepository cho đúng nguyên tắc kiến trúc phân lớp.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Alt thứ nhất đặt sau checkAvailability(): nhánh [xe khả dụng] → tiếp tục tạo booking; nhánh [xe không khả dụng] → trả thông báo lỗi cho UI. Alt thứ hai đặt sau processDeposit(): nhánh [thanh toán thành công] → xác nhận booking, cập nhật trạng thái xe = BOOKED; nhánh [thanh toán thất bại] → hủy booking, trả lỗi. Đánh giá: Vị trí đặt fragment chính xác. Em bổ sung thêm: ở nhánh [thanh toán thất bại] cần có thêm bước BookingRepository.updateStatus("CANCELLED") để rollback — AI đã bỏ qua bước này, nếu thiếu sẽ gây sai lệch dữ liệu giữa booking và thanh toán.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Nên đặt tên lifeline theo interface (ví dụ IBookingRepository) để thể hiện việc phụ thuộc vào abstraction; tên các message/method phải cụ thể như findById(), save(), updateStatus() — tránh ghi mơ hồ kiểu "truy vấn DB"; mỗi message chỉ nên đại diện cho một hành động DB, không gộp nhiều bước. Đánh giá: Phù hợp với nguyên lý Repository Pattern. Em áp dụng ngay: đổi tên lifeline BookingRepository thành IBookingRepository, và rà soát lại để mọi message gọi tới repository đều có tên method rõ ràng.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Luồng đề xuất: Staff nhập kết quả kiểm tra qua ReturnUI → InspectionController gọi InspectionService.evaluate() → trong opt [có hư hỏng]: gọi FeeService.calculateExtra() rồi PaymentRepository.save() → tiếp đến BookingService.complete() → BookingRepository.updateStatus("COMPLETED") → CarRepository.updateStatus("AVAILABLE") → trả kết quả về UI. Đánh giá: Luồng đầy đủ lớp và đúng trình tự. Em bổ sung thêm: sau bước updateStatus("COMPLETED") cần vẽ thêm message trả về (return message) từ Repository lên Service — đây là phần nhiều bạn dễ quên, khiến diagram bị thiếu tính khép kín.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: &lt;&lt;boundary&gt;&gt; dành cho các thành phần giao tiếp trực tiếp với actor (UI, API endpoint); &lt;&lt;control&gt;&gt; dành cho các lớp xử lý nghiệp vụ (Service, Controller); &lt;&lt;entity&gt;&gt; dành cho các lớp dữ liệu (Repository, Model/Entity). Trong AutoGo: BookingUI → boundary, BookingService → control, BookingRepository và Booking → entity. Đánh giá: Cách phân loại hợp lý. Em ghi chú thêm: thực tế trong Spring Boot, Controller đóng vai trò tiếp nhận request từ client nên về bản chất gần với &lt;&lt;boundary&gt;&gt; hơn — AI gán nó vào &lt;&lt;control&gt;&gt; chưa thật chuẩn, nhưng vẫn có thể tạm chấp nhận nếu áp dụng theo quy ước của Larman.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Đưa ra 6 tiêu chí: (1) đủ lifeline theo đúng kiến trúc phân lớp, (2) tên method cụ thể, không viết chung chung, (3) đúng loại mũi tên (đồng bộ/bất đồng bộ/trả về), (4) đặt alt fragment đúng vị trí, (5) có đầy đủ message trả về, (6) lifeline repository đặt tên theo interface. Đánh giá: Bộ tiêu chí khá toàn diện, bao quát những lỗi thường bị trừ điểm. Em bổ sung thêm 2 tiêu chí: (7) activation bar phải có độ dài tương ứng với thời gian thực thi của method (kết thúc đúng lúc method trả kết quả), (8) không để message đi ngược chiều thời gian giữa các lifeline — đây là 2 lỗi kỹ thuật thường gặp khi vẽ tay hoặc trên PlantUML.</t>
+  </si>
+  <si>
+    <t>"State diagram là gì? Phân biệt với sequence diagram và activity diagram?"</t>
+  </si>
+  <si>
+    <t>"Các phần tử cấu thành state diagram là gì? Mô tả ý nghĩa và ký hiệu vẽ của từng loại."</t>
+  </si>
+  <si>
+    <t>"Cú pháp nhãn của transition trong state diagram ra sao? event, guard, action khác nhau thế nào?"</t>
+  </si>
+  <si>
+    <t>"Thiết kế state diagram cho đối tượng Booking trong AutoGo, liệt kê đầy đủ các trạng thái và sự kiện chuyển đổi."</t>
+  </si>
+  <si>
+    <t>"Internal transition là gì? Với object Booking trong AutoGo, khi nào nên dùng internal transition thay vì self-transition?"</t>
+  </si>
+  <si>
+    <t>"Khi nào cần dùng composite state? Minh họa với object Payment trong AutoGo."</t>
+  </si>
+  <si>
+    <t>"Thiết kế state diagram cho object Car trong AutoGo. Trạng thái xe thay đổi như thế nào theo vòng đời của booking?"</t>
+  </si>
+  <si>
+    <t>"State diagram liên hệ với class diagram ra sao? Thuộc tính 'status' trong class Booking được ánh xạ như thế nào?"</t>
+  </si>
+  <si>
+    <t>"Trước khi nộp bài SWD392, cần dựa vào checklist nào để tự kiểm tra state diagram?"</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: State diagram (hay statechart) thể hiện vòng đời của một object thông qua các trạng thái và những sự kiện làm trạng thái thay đổi. Sự khác biệt: sequence diagram tập trung vào tương tác giữa nhiều object theo thời gian, activity diagram tập trung vào luồng công việc/quy trình, còn state diagram chỉ xoay quanh một object và các trạng thái nội tại của nó. Đánh giá: Giải thích chính xác, dễ hiểu. Em bổ sung thêm: loại diagram này đặc biệt phù hợp với các object có nhiều trạng thái phức tạp như Booking, Order, Payment — đây là use case điển hình mà AI chưa nêu ra.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Bao gồm: Initial Pseudostate (hình tròn đặc), Final State (vòng tròn lồng nhau với chấm đặc bên trong), State (hình chữ nhật bo góc), Transition (mũi tên kèm nhãn dạng event[guard]/action), Internal Transition (xử lý nội bộ trong state, không gây chuyển trạng thái), và Composite State (trạng thái chứa các sub-state). Đánh giá: Phù hợp chuẩn UML 2.x. Tuy nhiên AI bỏ qua Junction và Choice pseudostate — em tự bổ sung vì hai ký hiệu này thường xuất hiện khi transition có rẽ nhánh theo điều kiện.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Cú pháp chung là event [guard] / action. Trong đó event là sự kiện kích hoạt (ví dụ submitPayment), guard là điều kiện boolean đặt trong dấu ngoặc vuông (ví dụ [payment valid]), action là hành động được thực hiện khi transition xảy ra (ví dụ /sendConfirmation()). Cả ba phần đều có thể bỏ qua nhưng cần tối thiểu event hoặc guard. Đánh giá: Giải thích đầy đủ. Em ghi chú thêm lỗi thường gặp: guard phải là một biểu thức kiểm tra được tại thời điểm chạy, không phải là một lời gọi hành động — nhiều người nhầm viết [processPayment()] vào phần guard thay vì đặt nó ở phần action.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Đề xuất luồng: PENDING → [confirmBooking] → CONFIRMED → [payDeposit / payment valid] → DEPOSIT_PAID → [pickupCar] → ACTIVE → [returnCar] → RETURNED → [payRemaining] → COMPLETED. Nhánh hủy: từ PENDING hoặc CONFIRMED → [cancelBooking] → CANCELLED. Từ ACTIVE → [reportDamage] → DISPUTED. Đánh giá: Bao quát được các trạng thái nghiệp vụ chính. Rà soát lại em thấy còn thiếu trạng thái EXPIRED cho booking quá hạn chưa xác nhận — em bổ sung transition: PENDING → [timeout after 24h] → EXPIRED, để phản ánh đúng thực tế vận hành.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Internal transition xử lý một sự kiện ngay trong state hiện tại mà không thoát ra rồi vào lại (do đó không kích hoạt entry/exit action). Ngược lại, self-transition là thoát khỏi state rồi vào lại chính nó (có kích hoạt entry/exit). Ví dụ trong AutoGo: ở trạng thái CONFIRMED, sự kiện updateContactInfo không làm thay đổi trạng thái nên nên dùng internal transition. Đánh giá: Khái niệm chính xác. Em bổ sung thêm một trường hợp thực tế: ở trạng thái ACTIVE, sự kiện extendRentalPeriod cũng nên là internal transition vì booking vẫn giữ ACTIVE, chỉ thay đổi endDate — AI chưa đề cập đến case này.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Composite state phù hợp khi một trạng thái có logic xử lý nội bộ phức tạp, cần chia nhỏ thành các sub-state. Ví dụ: trạng thái PROCESSING của Payment có thể được tách thành các sub-state VALIDATING → CHARGING → NOTIFYING, có transition nội bộ giữa chúng. Đánh giá: Cách giải thích hợp lý. Em nhận thấy AI chưa nói đến history pseudostate (H) — dùng để ghi nhớ sub-state đang dừng trước khi rời composite state, để khi quay lại có thể tiếp tục đúng vị trí. Đây là điểm em ghi chú thêm vì thường gặp trong câu hỏi lý thuyết.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Đề xuất luồng: AVAILABLE → [bookingConfirmed] → RESERVED → [carPickedUp] → IN_USE → [carReturned] → INSPECTION → [inspectionPassed] → AVAILABLE; nhánh [inspectionFailed] → MAINTENANCE → [repairCompleted] → AVAILABLE. Ngoài ra còn nhánh AVAILABLE → [scheduledMaintenance] → MAINTENANCE. Đánh giá: Mối liên hệ giữa state của Car và Booking được thể hiện đúng bản chất domain. Em bổ sung thêm: cần có transition RESERVED → AVAILABLE khi booking bị CANCELLED hoặc EXPIRED — nếu thiếu case này, xe sẽ bị "kẹt" ở trạng thái RESERVED mãi mãi, điều mà AI đã bỏ sót.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Mỗi state trong state diagram tương ứng với một giá trị hợp lệ của thuộc tính status trong class. Mỗi transition tương ứng với một method làm thay đổi giá trị đó. Ví dụ: khi gọi confirmBooking() trong BookingService sẽ kích hoạt transition PENDING → CONFIRMED, đồng thời cập nhật booking.status = "CONFIRMED". Đánh giá: Mối liên kết giữa hai loại diagram được thể hiện rõ. Em bổ sung thêm góc nhìn triển khai: trong code Spring Boot, các giá trị trạng thái nên được định nghĩa dưới dạng enum BookingStatus thay vì kiểu String, vừa đảm bảo type-safe vừa khớp với state diagram — điều này AI chưa đề cập tới.</t>
+  </si>
+  <si>
+    <t>Phản hồi AI: Đưa ra 5 tiêu chí: (1) phải có initial pseudostate, (2) có tối thiểu một final state, (3) mọi state đều phải reachable được từ initial state, (4) nhãn transition tuân đúng cú pháp event[guard]/action, (5) không tồn tại state "cụt" — không có transition đi ra (ngoại trừ final state). Đánh giá: Bộ tiêu chí cơ bản đã khá đầy đủ. Em bổ sung thêm 3 tiêu chí: (6) rà soát lại guard condition để đảm bảo không bị viết nhầm thành action, (7) nếu có composite state thì bên trong cũng phải có initial pseudostate riêng, (8) đặt tên state theo SNAKE_CASE viết hoa để dễ phân biệt với tên event — đây là 3 lỗi kỹ thuật thường gặp khi vẽ trên PlantUML.</t>
   </si>
 </sst>
 </file>
@@ -1344,4 +1454,316 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09E46F54-5C02-4815-BBB2-036BA7D7340A}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="97.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>109</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEA5ADEE-A832-450B-B15F-1E3D0A90E75A}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="32" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="97.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6">
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6">
+        <v>3</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6">
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6">
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6">
+        <v>7</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>